<commit_message>
Update New Relic market reports - 2026-10-11 23:21:00
</commit_message>
<xml_diff>
--- a/output/b2b-kr.xlsx
+++ b/output/b2b-kr.xlsx
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>0</v>
+        <v>1478</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -614,7 +614,7 @@
         </is>
       </c>
       <c r="D6" s="6" t="n">
-        <v>0</v>
+        <v>1470</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
@@ -646,7 +646,7 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>0</v>
+        <v>1478</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="D9" s="6" t="n">
-        <v>0</v>
+        <v>1477</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
@@ -678,7 +678,7 @@
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0</v>
+        <v>1477</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-12 03:39:49
</commit_message>
<xml_diff>
--- a/output/b2b-kr.xlsx
+++ b/output/b2b-kr.xlsx
@@ -562,7 +562,7 @@
         </is>
       </c>
       <c r="D3" s="6" t="n">
-        <v>0</v>
+        <v>1779</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
@@ -806,7 +806,7 @@
         </is>
       </c>
       <c r="D18" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-12 11:31:33
</commit_message>
<xml_diff>
--- a/output/b2b-kr.xlsx
+++ b/output/b2b-kr.xlsx
@@ -562,7 +562,7 @@
         </is>
       </c>
       <c r="D3" s="6" t="n">
-        <v>1779</v>
+        <v>3633</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>1478</v>
+        <v>1507</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -646,7 +646,7 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>1478</v>
+        <v>1504</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-13 02:20:12
</commit_message>
<xml_diff>
--- a/output/b2b-kr.xlsx
+++ b/output/b2b-kr.xlsx
@@ -562,7 +562,7 @@
         </is>
       </c>
       <c r="D3" s="6" t="n">
-        <v>3633</v>
+        <v>2734</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>1571</v>
+        <v>3333</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -614,7 +614,7 @@
         </is>
       </c>
       <c r="D6" s="6" t="n">
-        <v>1470</v>
+        <v>1120</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
@@ -646,7 +646,7 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>1504</v>
+        <v>1672</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="D9" s="6" t="n">
-        <v>1477</v>
+        <v>1188</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
@@ -678,7 +678,7 @@
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>1477</v>
+        <v>1189</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-13 06:02:18
</commit_message>
<xml_diff>
--- a/output/b2b-kr.xlsx
+++ b/output/b2b-kr.xlsx
@@ -562,7 +562,7 @@
         </is>
       </c>
       <c r="D3" s="6" t="n">
-        <v>2734</v>
+        <v>474</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>3333</v>
+        <v>3315</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -646,7 +646,7 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>1672</v>
+        <v>1646</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
@@ -710,7 +710,7 @@
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-13 06:30:01
</commit_message>
<xml_diff>
--- a/output/b2b-kr.xlsx
+++ b/output/b2b-kr.xlsx
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>3315</v>
+        <v>3311</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -646,7 +646,7 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>1646</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-13 09:56:47
</commit_message>
<xml_diff>
--- a/output/b2b-kr.xlsx
+++ b/output/b2b-kr.xlsx
@@ -562,7 +562,7 @@
         </is>
       </c>
       <c r="D3" s="6" t="n">
-        <v>474</v>
+        <v>325</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>3311</v>
+        <v>3315</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-13 22:09:28
</commit_message>
<xml_diff>
--- a/output/b2b-kr.xlsx
+++ b/output/b2b-kr.xlsx
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>3334</v>
+        <v>2619</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -614,7 +614,7 @@
         </is>
       </c>
       <c r="D6" s="6" t="n">
-        <v>1120</v>
+        <v>1123</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
@@ -646,7 +646,7 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>1650</v>
+        <v>1185</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="D9" s="6" t="n">
-        <v>1188</v>
+        <v>1184</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
@@ -678,7 +678,7 @@
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>1189</v>
+        <v>1185</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-14 01:04:20
</commit_message>
<xml_diff>
--- a/output/b2b-kr.xlsx
+++ b/output/b2b-kr.xlsx
@@ -562,7 +562,7 @@
         </is>
       </c>
       <c r="D3" s="6" t="n">
-        <v>325</v>
+        <v>201</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>2619</v>
+        <v>2286</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -614,7 +614,7 @@
         </is>
       </c>
       <c r="D6" s="6" t="n">
-        <v>1123</v>
+        <v>1516</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
@@ -646,7 +646,7 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>1185</v>
+        <v>1193</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="D9" s="6" t="n">
-        <v>1184</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
@@ -678,7 +678,7 @@
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>1185</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-14 06:57:26
</commit_message>
<xml_diff>
--- a/output/b2b-kr.xlsx
+++ b/output/b2b-kr.xlsx
@@ -562,7 +562,7 @@
         </is>
       </c>
       <c r="D3" s="6" t="n">
-        <v>201</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
@@ -578,7 +578,7 @@
         </is>
       </c>
       <c r="D4" s="6" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>2286</v>
+        <v>2288</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -646,7 +646,7 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>1193</v>
+        <v>1189</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
@@ -710,7 +710,7 @@
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-14 12:39:31
</commit_message>
<xml_diff>
--- a/output/b2b-kr.xlsx
+++ b/output/b2b-kr.xlsx
@@ -562,7 +562,7 @@
         </is>
       </c>
       <c r="D3" s="6" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
@@ -578,7 +578,7 @@
         </is>
       </c>
       <c r="D4" s="6" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>2288</v>
+        <v>2289</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-14 21:10:26
</commit_message>
<xml_diff>
--- a/output/b2b-kr.xlsx
+++ b/output/b2b-kr.xlsx
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>2277</v>
+        <v>2910</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -646,7 +646,7 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>1189</v>
+        <v>1141</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-15 00:14:06
</commit_message>
<xml_diff>
--- a/output/b2b-kr.xlsx
+++ b/output/b2b-kr.xlsx
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>2910</v>
+        <v>3222</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -614,7 +614,7 @@
         </is>
       </c>
       <c r="D6" s="6" t="n">
-        <v>1516</v>
+        <v>1584</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
@@ -646,7 +646,7 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>1141</v>
+        <v>1584</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="D9" s="6" t="n">
-        <v>1142</v>
+        <v>1030</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
@@ -678,7 +678,7 @@
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>1142</v>
+        <v>1030</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-15 05:26:59
</commit_message>
<xml_diff>
--- a/output/b2b-kr.xlsx
+++ b/output/b2b-kr.xlsx
@@ -578,7 +578,7 @@
         </is>
       </c>
       <c r="D4" s="6" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
@@ -710,7 +710,7 @@
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-15 10:39:58
</commit_message>
<xml_diff>
--- a/output/b2b-kr.xlsx
+++ b/output/b2b-kr.xlsx
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>3222</v>
+        <v>3211</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -646,7 +646,7 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>1584</v>
+        <v>1585</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-15 22:49:30
</commit_message>
<xml_diff>
--- a/output/b2b-kr.xlsx
+++ b/output/b2b-kr.xlsx
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>3249</v>
+        <v>1952</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -614,7 +614,7 @@
         </is>
       </c>
       <c r="D6" s="6" t="n">
-        <v>1584</v>
+        <v>916</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
@@ -646,7 +646,7 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>1585</v>
+        <v>1477</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="D9" s="6" t="n">
-        <v>1030</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
@@ -678,7 +678,7 @@
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>1030</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-16 00:55:50
</commit_message>
<xml_diff>
--- a/output/b2b-kr.xlsx
+++ b/output/b2b-kr.xlsx
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>1952</v>
+        <v>2052</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -614,7 +614,7 @@
         </is>
       </c>
       <c r="D6" s="6" t="n">
-        <v>916</v>
+        <v>975</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="D9" s="6" t="n">
-        <v>1390</v>
+        <v>1477</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
@@ -678,7 +678,7 @@
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>1390</v>
+        <v>1477</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-16 05:20:58
</commit_message>
<xml_diff>
--- a/output/b2b-kr.xlsx
+++ b/output/b2b-kr.xlsx
@@ -578,7 +578,7 @@
         </is>
       </c>
       <c r="D4" s="6" t="n">
-        <v>14</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>2052</v>
+        <v>2074</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -646,7 +646,7 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>1477</v>
+        <v>1492</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
@@ -710,7 +710,7 @@
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-16 10:26:59
</commit_message>
<xml_diff>
--- a/output/b2b-kr.xlsx
+++ b/output/b2b-kr.xlsx
@@ -578,7 +578,7 @@
         </is>
       </c>
       <c r="D4" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>2074</v>
+        <v>2134</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -646,7 +646,7 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>1492</v>
+        <v>1505</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-16 22:22:48
</commit_message>
<xml_diff>
--- a/output/b2b-kr.xlsx
+++ b/output/b2b-kr.xlsx
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>2133</v>
+        <v>754</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -614,7 +614,7 @@
         </is>
       </c>
       <c r="D6" s="6" t="n">
-        <v>975</v>
+        <v>590</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
@@ -646,7 +646,7 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>1505</v>
+        <v>29</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="D9" s="6" t="n">
-        <v>1477</v>
+        <v>881</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
@@ -678,7 +678,7 @@
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>1477</v>
+        <v>881</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-17 00:56:55
</commit_message>
<xml_diff>
--- a/output/b2b-kr.xlsx
+++ b/output/b2b-kr.xlsx
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>754</v>
+        <v>139</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -614,7 +614,7 @@
         </is>
       </c>
       <c r="D6" s="6" t="n">
-        <v>590</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="D9" s="6" t="n">
-        <v>881</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
@@ -678,7 +678,7 @@
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>881</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
@@ -806,7 +806,7 @@
         </is>
       </c>
       <c r="D18" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-17 05:18:26
</commit_message>
<xml_diff>
--- a/output/b2b-kr.xlsx
+++ b/output/b2b-kr.xlsx
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>139</v>
+        <v>125</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -646,7 +646,7 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>29</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-17 09:58:21
</commit_message>
<xml_diff>
--- a/output/b2b-kr.xlsx
+++ b/output/b2b-kr.xlsx
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>125</v>
+        <v>54</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -646,7 +646,7 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-18 22:08:34
</commit_message>
<xml_diff>
--- a/output/b2b-kr.xlsx
+++ b/output/b2b-kr.xlsx
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>3</v>
+        <v>1842</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -614,7 +614,7 @@
         </is>
       </c>
       <c r="D6" s="6" t="n">
-        <v>0</v>
+        <v>1005</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
@@ -646,7 +646,7 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>0</v>
+        <v>206</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="D9" s="6" t="n">
-        <v>0</v>
+        <v>1006</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
@@ -678,7 +678,7 @@
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>0</v>
+        <v>1006</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-19 00:40:03
</commit_message>
<xml_diff>
--- a/output/b2b-kr.xlsx
+++ b/output/b2b-kr.xlsx
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>1842</v>
+        <v>1989</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -614,7 +614,7 @@
         </is>
       </c>
       <c r="D6" s="6" t="n">
-        <v>1005</v>
+        <v>1182</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="D9" s="6" t="n">
-        <v>1006</v>
+        <v>1183</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
@@ -678,7 +678,7 @@
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>1006</v>
+        <v>1183</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
@@ -806,7 +806,7 @@
         </is>
       </c>
       <c r="D18" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-19 05:34:11
</commit_message>
<xml_diff>
--- a/output/b2b-kr.xlsx
+++ b/output/b2b-kr.xlsx
@@ -562,7 +562,7 @@
         </is>
       </c>
       <c r="D3" s="6" t="n">
-        <v>9</v>
+        <v>83</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>1989</v>
+        <v>2013</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -646,7 +646,7 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>206</v>
+        <v>217</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-19 11:45:58
</commit_message>
<xml_diff>
--- a/output/b2b-kr.xlsx
+++ b/output/b2b-kr.xlsx
@@ -562,7 +562,7 @@
         </is>
       </c>
       <c r="D3" s="6" t="n">
-        <v>83</v>
+        <v>136</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>2013</v>
+        <v>2015</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-19 18:06:19
</commit_message>
<xml_diff>
--- a/output/b2b-kr.xlsx
+++ b/output/b2b-kr.xlsx
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>2015</v>
+        <v>2016</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="D9" s="6" t="n">
-        <v>1183</v>
+        <v>1184</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
@@ -678,7 +678,7 @@
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>1183</v>
+        <v>1184</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
@@ -710,7 +710,7 @@
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-19 22:44:13
</commit_message>
<xml_diff>
--- a/output/b2b-kr.xlsx
+++ b/output/b2b-kr.xlsx
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>2016</v>
+        <v>2302</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -614,7 +614,7 @@
         </is>
       </c>
       <c r="D6" s="6" t="n">
-        <v>1182</v>
+        <v>642</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
@@ -646,7 +646,7 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>217</v>
+        <v>1077</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="D9" s="6" t="n">
-        <v>1184</v>
+        <v>657</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
@@ -678,7 +678,7 @@
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>1184</v>
+        <v>657</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-20 01:25:28
</commit_message>
<xml_diff>
--- a/output/b2b-kr.xlsx
+++ b/output/b2b-kr.xlsx
@@ -562,7 +562,7 @@
         </is>
       </c>
       <c r="D3" s="6" t="n">
-        <v>136</v>
+        <v>140</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>2302</v>
+        <v>2866</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -614,7 +614,7 @@
         </is>
       </c>
       <c r="D6" s="6" t="n">
-        <v>642</v>
+        <v>1207</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="D9" s="6" t="n">
-        <v>657</v>
+        <v>1176</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
@@ -678,7 +678,7 @@
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>657</v>
+        <v>1177</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-20 06:58:35
</commit_message>
<xml_diff>
--- a/output/b2b-kr.xlsx
+++ b/output/b2b-kr.xlsx
@@ -562,7 +562,7 @@
         </is>
       </c>
       <c r="D3" s="6" t="n">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
@@ -646,7 +646,7 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>1077</v>
+        <v>1099</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-20 12:34:37
</commit_message>
<xml_diff>
--- a/output/b2b-kr.xlsx
+++ b/output/b2b-kr.xlsx
@@ -562,7 +562,7 @@
         </is>
       </c>
       <c r="D3" s="6" t="n">
-        <v>141</v>
+        <v>116</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>2866</v>
+        <v>2865</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-20 17:41:56
</commit_message>
<xml_diff>
--- a/output/b2b-kr.xlsx
+++ b/output/b2b-kr.xlsx
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>2865</v>
+        <v>2891</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="D9" s="6" t="n">
-        <v>1176</v>
+        <v>1175</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
@@ -678,7 +678,7 @@
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>1177</v>
+        <v>1176</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
@@ -710,7 +710,7 @@
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-20 21:06:25
</commit_message>
<xml_diff>
--- a/output/b2b-kr.xlsx
+++ b/output/b2b-kr.xlsx
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>2891</v>
+        <v>2914</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -646,7 +646,7 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>1099</v>
+        <v>1426</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-21 00:18:15
</commit_message>
<xml_diff>
--- a/output/b2b-kr.xlsx
+++ b/output/b2b-kr.xlsx
@@ -562,7 +562,7 @@
         </is>
       </c>
       <c r="D3" s="6" t="n">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>2914</v>
+        <v>2152</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -614,7 +614,7 @@
         </is>
       </c>
       <c r="D6" s="6" t="n">
-        <v>1207</v>
+        <v>1543</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
@@ -646,7 +646,7 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>1426</v>
+        <v>1576</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="D9" s="6" t="n">
-        <v>1175</v>
+        <v>1017</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
@@ -678,7 +678,7 @@
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>1176</v>
+        <v>1017</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-21 05:37:11
</commit_message>
<xml_diff>
--- a/output/b2b-kr.xlsx
+++ b/output/b2b-kr.xlsx
@@ -562,7 +562,7 @@
         </is>
       </c>
       <c r="D3" s="6" t="n">
-        <v>103</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>2152</v>
+        <v>2134</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -646,7 +646,7 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>1576</v>
+        <v>1551</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-21 10:57:57
</commit_message>
<xml_diff>
--- a/output/b2b-kr.xlsx
+++ b/output/b2b-kr.xlsx
@@ -562,7 +562,7 @@
         </is>
       </c>
       <c r="D3" s="6" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>2134</v>
+        <v>2157</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -646,7 +646,7 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>1551</v>
+        <v>1550</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-21 22:57:26
</commit_message>
<xml_diff>
--- a/output/b2b-kr.xlsx
+++ b/output/b2b-kr.xlsx
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>2165</v>
+        <v>3133</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -614,7 +614,7 @@
         </is>
       </c>
       <c r="D6" s="6" t="n">
-        <v>1543</v>
+        <v>899</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
@@ -646,7 +646,7 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>1550</v>
+        <v>1733</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="D9" s="6" t="n">
-        <v>1017</v>
+        <v>458</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
@@ -678,7 +678,7 @@
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>1017</v>
+        <v>458</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-22 01:12:55
</commit_message>
<xml_diff>
--- a/output/b2b-kr.xlsx
+++ b/output/b2b-kr.xlsx
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>3133</v>
+        <v>3698</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -614,7 +614,7 @@
         </is>
       </c>
       <c r="D6" s="6" t="n">
-        <v>899</v>
+        <v>1196</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
@@ -646,7 +646,7 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>1733</v>
+        <v>1740</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="D9" s="6" t="n">
-        <v>458</v>
+        <v>787</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
@@ -678,7 +678,7 @@
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>458</v>
+        <v>787</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-22 06:56:10
</commit_message>
<xml_diff>
--- a/output/b2b-kr.xlsx
+++ b/output/b2b-kr.xlsx
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>3698</v>
+        <v>3675</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -646,7 +646,7 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>1740</v>
+        <v>1739</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-22 17:48:09
</commit_message>
<xml_diff>
--- a/output/b2b-kr.xlsx
+++ b/output/b2b-kr.xlsx
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>3675</v>
+        <v>3685</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="D17" s="6" t="n">
-        <v>542</v>
+        <v>354</v>
       </c>
     </row>
     <row r="18" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-22 21:03:59
</commit_message>
<xml_diff>
--- a/output/b2b-kr.xlsx
+++ b/output/b2b-kr.xlsx
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>3685</v>
+        <v>3412</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -646,7 +646,7 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>1739</v>
+        <v>1938</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-23 00:18:58
</commit_message>
<xml_diff>
--- a/output/b2b-kr.xlsx
+++ b/output/b2b-kr.xlsx
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>3412</v>
+        <v>2333</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -614,7 +614,7 @@
         </is>
       </c>
       <c r="D6" s="6" t="n">
-        <v>1196</v>
+        <v>1661</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
@@ -646,7 +646,7 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>1938</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="D9" s="6" t="n">
-        <v>787</v>
+        <v>1117</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
@@ -678,7 +678,7 @@
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>787</v>
+        <v>1117</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-23 01:32:02
</commit_message>
<xml_diff>
--- a/output/b2b-kr.xlsx
+++ b/output/b2b-kr.xlsx
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>2333</v>
+        <v>2328</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -646,7 +646,7 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>1674</v>
+        <v>1665</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-23 05:38:14
</commit_message>
<xml_diff>
--- a/output/b2b-kr.xlsx
+++ b/output/b2b-kr.xlsx
@@ -646,7 +646,7 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>1665</v>
+        <v>1669</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
@@ -710,7 +710,7 @@
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-23 15:35:09
</commit_message>
<xml_diff>
--- a/output/b2b-kr.xlsx
+++ b/output/b2b-kr.xlsx
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="D17" s="6" t="n">
-        <v>354</v>
+        <v>542</v>
       </c>
     </row>
     <row r="18" ht="22" customHeight="1">
@@ -806,7 +806,7 @@
         </is>
       </c>
       <c r="D18" s="6" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-23 22:48:40
</commit_message>
<xml_diff>
--- a/output/b2b-kr.xlsx
+++ b/output/b2b-kr.xlsx
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>2290</v>
+        <v>400</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -614,7 +614,7 @@
         </is>
       </c>
       <c r="D6" s="6" t="n">
-        <v>1661</v>
+        <v>270</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
@@ -646,7 +646,7 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>1669</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="D9" s="6" t="n">
-        <v>1117</v>
+        <v>186</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
@@ -678,7 +678,7 @@
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>1117</v>
+        <v>186</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
@@ -806,7 +806,7 @@
         </is>
       </c>
       <c r="D18" s="6" t="n">
-        <v>4</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-24 01:18:16
</commit_message>
<xml_diff>
--- a/output/b2b-kr.xlsx
+++ b/output/b2b-kr.xlsx
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>400</v>
+        <v>48</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -614,7 +614,7 @@
         </is>
       </c>
       <c r="D6" s="6" t="n">
-        <v>270</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="D9" s="6" t="n">
-        <v>186</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
@@ -678,7 +678,7 @@
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>186</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
@@ -806,7 +806,7 @@
         </is>
       </c>
       <c r="D18" s="6" t="n">
-        <v>55</v>
+        <v>205</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-24 06:45:03
</commit_message>
<xml_diff>
--- a/output/b2b-kr.xlsx
+++ b/output/b2b-kr.xlsx
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>48</v>
+        <v>40</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -630,7 +630,7 @@
         </is>
       </c>
       <c r="D7" s="6" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
@@ -646,7 +646,7 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
@@ -710,7 +710,7 @@
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
@@ -806,7 +806,7 @@
         </is>
       </c>
       <c r="D18" s="6" t="n">
-        <v>205</v>
+        <v>532</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update New Relic market reports - 2026-10-24 11:46:15
</commit_message>
<xml_diff>
--- a/output/b2b-kr.xlsx
+++ b/output/b2b-kr.xlsx
@@ -630,7 +630,7 @@
         </is>
       </c>
       <c r="D7" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
@@ -806,7 +806,7 @@
         </is>
       </c>
       <c r="D18" s="6" t="n">
-        <v>532</v>
+        <v>833</v>
       </c>
     </row>
   </sheetData>

</xml_diff>